<commit_message>
Daily EOD data and reports for 2026-08-18
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260818.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260818.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.612</v>
+        <v>1.62</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.017</v>
+        <v>0.025</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1.07%</t>
+          <t>1.57%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>246927.77</v>
+        <v>248153.22</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>2604.08</v>
+        <v>3829.53</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.315</v>
+        <v>2.31</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.015</v>
+        <v>0.01</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.65%</t>
+          <t>0.43%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>162050</v>
+        <v>161700</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>1050</v>
+        <v>700</v>
       </c>
     </row>
     <row r="6">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>64.27</v>
+        <v>64.205</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>2.07</v>
+        <v>2.005</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3.33%</t>
+          <t>3.22%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>11065</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>711147.55</v>
+        <v>710428.3199999999</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>22904.55</v>
+        <v>22185.32</v>
       </c>
     </row>
     <row r="8">
@@ -596,24 +596,24 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>-0.003</v>
+        <v>0</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
         <v>44090</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>0</v>
+        <v>132.27</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-132.27</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -623,14 +623,14 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>163.31</v>
+        <v>163.19</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-1.69</v>
+        <v>-1.81</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-1.02%</t>
+          <t>-1.10%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>154.36</v>
+        <v>155.52</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>19.76</v>
+        <v>20.92</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>14.68%</t>
+          <t>15.54%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>617440</v>
+        <v>622080</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>79040</v>
+        <v>83680</v>
       </c>
     </row>
     <row r="12">
@@ -758,24 +758,24 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0</v>
+        <v>0.13</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>-0.13</v>
+        <v>0</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
         <v>9412</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>0</v>
+        <v>1223.56</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>-1223.56</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -785,24 +785,24 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>-0.102</v>
+        <v>-0.002</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>-1.96%</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
         <v>6000</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>-612</v>
+        <v>-12</v>
       </c>
     </row>
     <row r="16">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>34.615</v>
+        <v>34.62</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>-0.455</v>
+        <v>-0.45</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-1.30%</t>
+          <t>-1.28%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>33.07</v>
+        <v>33.09</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.22</v>
+        <v>0.24</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0.67%</t>
+          <t>0.73%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>42594.16</v>
+        <v>42619.92</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>283.36</v>
+        <v>309.12</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1864520.95</v>
+        <v>1871298.77</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>101077.71</v>
+        <v>107855.52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>